<commit_message>
fix(workspace): repair blank OOXML templates and editor /ds base URL
Incomplete blank.docx (missing document.xml.rels/styles) made DocumentServer
show Download failed after the ribbon loaded; also set documentServerUrl and
ALLOW_META_IP_ADDRESS for compose-internal downloads.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/indobase-suite/bridge/templates/blank.xlsx
+++ b/indobase-suite/bridge/templates/blank.xlsx
@@ -7,6 +7,35 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="0" uniqueCount="0"/>
+</file>
+
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="1">
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+  </fonts>
+  <fills count="1">
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border/>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf/>
+  </cellStyleXfs>
+  <cellXfs count="1">
+    <xf xfId="0"/>
+  </cellXfs>
+</styleSheet>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetData/>

</xml_diff>